<commit_message>
Cambios excel lapiz stock
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucil\Desktop\rmkits-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41261EF3-F30C-446C-835B-CD88391E9FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908B6534-5472-46C5-BCCC-6131A4C05627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="17380" windowHeight="7360" xr2:uid="{C4B6B2E4-7AFF-45F0-BE4D-6E6AB0ED2031}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="17390" windowHeight="7370" xr2:uid="{C4B6B2E4-7AFF-45F0-BE4D-6E6AB0ED2031}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1721,7 +1721,7 @@
         <v>6</v>
       </c>
       <c r="G12" s="5">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>43</v>

</xml_diff>

<commit_message>
Cambios excel agregue productos
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucil\Desktop\rmkits-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD924234-E42B-4922-AC23-8A7E77B650CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25564EA4-A796-44CA-913D-60037C28D03E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="0" windowWidth="18780" windowHeight="10200" xr2:uid="{C4B6B2E4-7AFF-45F0-BE4D-6E6AB0ED2031}"/>
+    <workbookView xWindow="150" yWindow="1460" windowWidth="8860" windowHeight="9820" xr2:uid="{C4B6B2E4-7AFF-45F0-BE4D-6E6AB0ED2031}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="338">
   <si>
     <t>codigo</t>
   </si>
@@ -90,9 +90,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>Corrector liquido Filgo 012 (unidad)</t>
-  </si>
-  <si>
     <t>Cinta correctora Filgo 12mts</t>
   </si>
   <si>
@@ -810,9 +807,6 @@
     <t>Papel glase fluo sobre x5 hojas</t>
   </si>
   <si>
-    <t>Lapiz negro grafito Filgo HB (unidad)</t>
-  </si>
-  <si>
     <t>Cinta de papel 24mm</t>
   </si>
   <si>
@@ -934,6 +928,126 @@
   </si>
   <si>
     <t>Repuesto Canson N°5 Color x6 hojas Triunfante</t>
+  </si>
+  <si>
+    <t>A0137</t>
+  </si>
+  <si>
+    <t>A0138</t>
+  </si>
+  <si>
+    <t>A0139</t>
+  </si>
+  <si>
+    <t>A0140</t>
+  </si>
+  <si>
+    <t>A0141</t>
+  </si>
+  <si>
+    <t>A0142</t>
+  </si>
+  <si>
+    <t>Puntero Láser colores pastel</t>
+  </si>
+  <si>
+    <t>Avion Planeador de Telgopor</t>
+  </si>
+  <si>
+    <t>Pollito Kawaii con ganchito</t>
+  </si>
+  <si>
+    <t>Soga de saltar infantil</t>
+  </si>
+  <si>
+    <t>Escarapela Argentina Moño</t>
+  </si>
+  <si>
+    <t>Escarapela Argentina Circular</t>
+  </si>
+  <si>
+    <t>Bandera Plástica 15x25 Argentina</t>
+  </si>
+  <si>
+    <t>A0143</t>
+  </si>
+  <si>
+    <t>A0144</t>
+  </si>
+  <si>
+    <t>A0145</t>
+  </si>
+  <si>
+    <t>A0146</t>
+  </si>
+  <si>
+    <t>A0147</t>
+  </si>
+  <si>
+    <t>Gusano Extensible</t>
+  </si>
+  <si>
+    <t>Lapiceras 4 colores en 1 unicornio</t>
+  </si>
+  <si>
+    <t>Silbatos</t>
+  </si>
+  <si>
+    <t>Portasube Colgante Colores Surtidos</t>
+  </si>
+  <si>
+    <t>Portasube Colgante Color Negro</t>
+  </si>
+  <si>
+    <t>A0148</t>
+  </si>
+  <si>
+    <t>Magic Snake Juego Ingenio</t>
+  </si>
+  <si>
+    <t>Masas Saltarinas PlayLife bolsa x15 masas</t>
+  </si>
+  <si>
+    <t>Capibara Squishy Yoyo con luz</t>
+  </si>
+  <si>
+    <t>Pelotitas Saltarinas</t>
+  </si>
+  <si>
+    <t>Tubo Plegable Antiestres con Luz</t>
+  </si>
+  <si>
+    <t>Copa del Mundo Alcancia Plastica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pulseras Luminosas </t>
+  </si>
+  <si>
+    <t>A0149</t>
+  </si>
+  <si>
+    <t>A0150</t>
+  </si>
+  <si>
+    <t>A0151</t>
+  </si>
+  <si>
+    <t>A0152</t>
+  </si>
+  <si>
+    <t>A0153</t>
+  </si>
+  <si>
+    <t>A0154</t>
+  </si>
+  <si>
+    <t>A0155</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lapiz negro grafito Filgo HB </t>
+  </si>
+  <si>
+    <t>Corrector liquido Filgo 012</t>
   </si>
 </sst>
 </file>
@@ -961,15 +1075,21 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1031,11 +1151,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1062,6 +1191,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1376,7 +1521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B0D8A5A-108C-466C-953C-70B57E87E4C5}">
-  <dimension ref="A1:I137"/>
+  <dimension ref="A1:I156"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.1796875" customWidth="1"/>
@@ -1411,7 +1556,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -1419,7 +1564,7 @@
         <v>8</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>258</v>
+        <v>336</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>16</v>
@@ -1440,7 +1585,7 @@
         <v>12</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -1448,7 +1593,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>18</v>
+        <v>337</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>17</v>
@@ -1469,7 +1614,7 @@
         <v>13</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -1477,7 +1622,7 @@
         <v>10</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>17</v>
@@ -1498,7 +1643,7 @@
         <v>14</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -1506,7 +1651,7 @@
         <v>11</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>17</v>
@@ -1527,15 +1672,15 @@
         <v>15</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>17</v>
@@ -1553,18 +1698,18 @@
         <v>500</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>17</v>
@@ -1582,18 +1727,18 @@
         <v>5000</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>17</v>
@@ -1611,18 +1756,18 @@
         <v>5000</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>17</v>
@@ -1640,18 +1785,18 @@
         <v>1500</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>17</v>
@@ -1669,18 +1814,18 @@
         <v>1500</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>17</v>
@@ -1698,18 +1843,18 @@
         <v>2400</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>17</v>
@@ -1727,18 +1872,18 @@
         <v>0</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>17</v>
@@ -1756,18 +1901,18 @@
         <v>120</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>17</v>
@@ -1785,18 +1930,18 @@
         <v>0</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>17</v>
@@ -1814,18 +1959,18 @@
         <v>2000</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>17</v>
@@ -1843,18 +1988,18 @@
         <v>2000</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>17</v>
@@ -1876,15 +2021,15 @@
         <v>A0018.jpg</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>17</v>
@@ -1906,15 +2051,15 @@
         <v>A0019.jpg</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>17</v>
@@ -1936,15 +2081,15 @@
         <v>A0020.jpg</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>17</v>
@@ -1966,15 +2111,15 @@
         <v>A0021.jpg</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>17</v>
@@ -1996,15 +2141,15 @@
         <v>A0045.jpg</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>17</v>
@@ -2026,15 +2171,15 @@
         <v>A0016.jpg</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>17</v>
@@ -2056,15 +2201,15 @@
         <v>A0017.jpg</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>17</v>
@@ -2086,15 +2231,15 @@
         <v>A0022.jpg</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>17</v>
@@ -2116,15 +2261,15 @@
         <v>A0023.jpg</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>17</v>
@@ -2146,15 +2291,15 @@
         <v>A0024.jpg</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>17</v>
@@ -2176,15 +2321,15 @@
         <v>A0025.jpg</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>17</v>
@@ -2206,15 +2351,15 @@
         <v>A0026.jpg</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>17</v>
@@ -2236,15 +2381,15 @@
         <v>A0027.jpg</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>17</v>
@@ -2266,15 +2411,15 @@
         <v>A0028.jpg</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>17</v>
@@ -2296,15 +2441,15 @@
         <v>A0029.jpg</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>17</v>
@@ -2326,15 +2471,15 @@
         <v>A0030.jpg</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>17</v>
@@ -2356,15 +2501,15 @@
         <v>A0031.jpg</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>17</v>
@@ -2386,15 +2531,15 @@
         <v>A0032.jpg</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>17</v>
@@ -2416,15 +2561,15 @@
         <v>A0033.jpg</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>17</v>
@@ -2446,15 +2591,15 @@
         <v>A0034.jpg</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>17</v>
@@ -2476,15 +2621,15 @@
         <v>A0035.jpg</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>17</v>
@@ -2506,15 +2651,15 @@
         <v>A0036.jpg</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>17</v>
@@ -2536,15 +2681,15 @@
         <v>A0037.jpg</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>17</v>
@@ -2566,15 +2711,15 @@
         <v>A0038.jpg</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>17</v>
@@ -2596,15 +2741,15 @@
         <v>A0039.jpg</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>17</v>
@@ -2626,15 +2771,15 @@
         <v>A0040.jpg</v>
       </c>
       <c r="I42" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>17</v>
@@ -2656,15 +2801,15 @@
         <v>A0041.jpg</v>
       </c>
       <c r="I43" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>17</v>
@@ -2686,15 +2831,15 @@
         <v>A0042.jpg</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5">
@@ -2714,15 +2859,15 @@
         <v>A0133.jpg</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5">
@@ -2742,15 +2887,15 @@
         <v>A0134.jpg</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>17</v>
@@ -2772,15 +2917,15 @@
         <v>A0043.jpg</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>17</v>
@@ -2802,15 +2947,15 @@
         <v>A0044.jpg</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C49" s="6"/>
       <c r="D49" s="7">
@@ -2830,15 +2975,15 @@
         <v>A0046.jpg</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="7">
@@ -2858,15 +3003,15 @@
         <v>A0047.jpg</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>17</v>
@@ -2888,15 +3033,15 @@
         <v>A0048.jpg</v>
       </c>
       <c r="I51" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>17</v>
@@ -2918,15 +3063,15 @@
         <v>A0049.jpg</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>17</v>
@@ -2948,15 +3093,15 @@
         <v>A0050.jpg</v>
       </c>
       <c r="I53" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>17</v>
@@ -2978,15 +3123,15 @@
         <v>A0051.jpg</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>17</v>
@@ -3008,15 +3153,15 @@
         <v>A0052.jpg</v>
       </c>
       <c r="I55" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>17</v>
@@ -3038,15 +3183,15 @@
         <v>A0053.jpg</v>
       </c>
       <c r="I56" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>17</v>
@@ -3068,15 +3213,15 @@
         <v>A0054.jpg</v>
       </c>
       <c r="I57" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>17</v>
@@ -3098,15 +3243,15 @@
         <v>A0055.jpg</v>
       </c>
       <c r="I58" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="26" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>17</v>
@@ -3128,15 +3273,15 @@
         <v>A0056.jpg</v>
       </c>
       <c r="I59" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>17</v>
@@ -3158,15 +3303,15 @@
         <v>A0057.jpg</v>
       </c>
       <c r="I60" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>17</v>
@@ -3188,15 +3333,15 @@
         <v>A0058.jpg</v>
       </c>
       <c r="I61" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>17</v>
@@ -3218,15 +3363,15 @@
         <v>A0059.jpg</v>
       </c>
       <c r="I62" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>17</v>
@@ -3248,15 +3393,15 @@
         <v>A0060.jpg</v>
       </c>
       <c r="I63" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>17</v>
@@ -3278,15 +3423,15 @@
         <v>A0061.jpg</v>
       </c>
       <c r="I64" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>17</v>
@@ -3308,15 +3453,15 @@
         <v>A0062.jpg</v>
       </c>
       <c r="I65" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>17</v>
@@ -3338,15 +3483,15 @@
         <v>A0063.jpg</v>
       </c>
       <c r="I66" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>17</v>
@@ -3368,15 +3513,15 @@
         <v>A0064.jpg</v>
       </c>
       <c r="I67" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>17</v>
@@ -3398,15 +3543,15 @@
         <v>A0065.jpg</v>
       </c>
       <c r="I68" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>17</v>
@@ -3428,15 +3573,15 @@
         <v>A0066.jpg</v>
       </c>
       <c r="I69" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>17</v>
@@ -3458,15 +3603,15 @@
         <v>A0067.jpg</v>
       </c>
       <c r="I70" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>17</v>
@@ -3488,15 +3633,15 @@
         <v>A0068.jpg</v>
       </c>
       <c r="I71" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>17</v>
@@ -3518,15 +3663,15 @@
         <v>A0069.jpg</v>
       </c>
       <c r="I72" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>17</v>
@@ -3548,15 +3693,15 @@
         <v>A0070.jpg</v>
       </c>
       <c r="I73" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>17</v>
@@ -3578,15 +3723,15 @@
         <v>A0071.jpg</v>
       </c>
       <c r="I74" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="75" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>17</v>
@@ -3608,15 +3753,15 @@
         <v>A0072.jpg</v>
       </c>
       <c r="I75" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>17</v>
@@ -3638,15 +3783,15 @@
         <v>A0073.jpg</v>
       </c>
       <c r="I76" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>17</v>
@@ -3668,15 +3813,15 @@
         <v>A0074.jpg</v>
       </c>
       <c r="I77" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>17</v>
@@ -3698,15 +3843,15 @@
         <v>A0075.jpg</v>
       </c>
       <c r="I78" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>17</v>
@@ -3728,15 +3873,15 @@
         <v>A0076.jpg</v>
       </c>
       <c r="I79" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>17</v>
@@ -3758,15 +3903,15 @@
         <v>A0077.jpg</v>
       </c>
       <c r="I80" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="81" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>17</v>
@@ -3788,15 +3933,15 @@
         <v>A0078.jpg</v>
       </c>
       <c r="I81" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="82" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>17</v>
@@ -3814,19 +3959,19 @@
         <v>120</v>
       </c>
       <c r="H82" t="str">
-        <f t="shared" ref="H82:H137" si="1">_xlfn.CONCAT(A82,".jpg")</f>
+        <f t="shared" ref="H82:H145" si="1">_xlfn.CONCAT(A82,".jpg")</f>
         <v>A0135.jpg</v>
       </c>
       <c r="I82" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="83" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>17</v>
@@ -3848,15 +3993,15 @@
         <v>A0079.jpg</v>
       </c>
       <c r="I83" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="84" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>17</v>
@@ -3878,15 +4023,15 @@
         <v>A0080.jpg</v>
       </c>
       <c r="I84" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="85" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>17</v>
@@ -3908,15 +4053,15 @@
         <v>A0081.jpg</v>
       </c>
       <c r="I85" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="86" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>17</v>
@@ -3938,15 +4083,15 @@
         <v>A0082.jpg</v>
       </c>
       <c r="I86" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="87" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>17</v>
@@ -3968,15 +4113,15 @@
         <v>A0083.jpg</v>
       </c>
       <c r="I87" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="88" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B88" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>17</v>
@@ -3998,15 +4143,15 @@
         <v>A0084.jpg</v>
       </c>
       <c r="I88" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="89" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>17</v>
@@ -4028,15 +4173,15 @@
         <v>A0085.jpg</v>
       </c>
       <c r="I89" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="90" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>17</v>
@@ -4058,15 +4203,15 @@
         <v>A0086.jpg</v>
       </c>
       <c r="I90" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="91" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>17</v>
@@ -4088,15 +4233,15 @@
         <v>A0087.jpg</v>
       </c>
       <c r="I91" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="92" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>17</v>
@@ -4118,15 +4263,15 @@
         <v>A0088.jpg</v>
       </c>
       <c r="I92" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="93" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C93" s="1"/>
       <c r="D93" s="2">
@@ -4146,15 +4291,15 @@
         <v>A0089.jpg</v>
       </c>
       <c r="I93" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="94" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C94" s="1"/>
       <c r="D94" s="2">
@@ -4174,15 +4319,15 @@
         <v>A0090.jpg</v>
       </c>
       <c r="I94" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="95" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C95" s="1"/>
       <c r="D95" s="2">
@@ -4202,15 +4347,15 @@
         <v>A0091.jpg</v>
       </c>
       <c r="I95" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="96" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C96" s="1"/>
       <c r="D96" s="2">
@@ -4230,15 +4375,15 @@
         <v>A0092.jpg</v>
       </c>
       <c r="I96" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="97" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C97" s="1"/>
       <c r="D97" s="2">
@@ -4258,15 +4403,15 @@
         <v>A0093.jpg</v>
       </c>
       <c r="I97" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="98" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C98" s="1"/>
       <c r="D98" s="2">
@@ -4286,15 +4431,15 @@
         <v>A0094.jpg</v>
       </c>
       <c r="I98" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="99" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C99" s="1"/>
       <c r="D99" s="2">
@@ -4314,15 +4459,15 @@
         <v>A0095.jpg</v>
       </c>
       <c r="I99" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="100" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>17</v>
@@ -4344,15 +4489,15 @@
         <v>A0096.jpg</v>
       </c>
       <c r="I100" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>17</v>
@@ -4374,15 +4519,15 @@
         <v>A0097.jpg</v>
       </c>
       <c r="I101" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="102" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>17</v>
@@ -4404,15 +4549,15 @@
         <v>A0098.jpg</v>
       </c>
       <c r="I102" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="103" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>17</v>
@@ -4434,15 +4579,15 @@
         <v>A0099.jpg</v>
       </c>
       <c r="I103" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="104" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>17</v>
@@ -4464,15 +4609,15 @@
         <v>A0100.jpg</v>
       </c>
       <c r="I104" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="105" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>17</v>
@@ -4494,15 +4639,15 @@
         <v>A0101.jpg</v>
       </c>
       <c r="I105" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="106" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>17</v>
@@ -4524,15 +4669,15 @@
         <v>A0102.jpg</v>
       </c>
       <c r="I106" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="107" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>17</v>
@@ -4554,15 +4699,15 @@
         <v>A0103.jpg</v>
       </c>
       <c r="I107" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="108" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>17</v>
@@ -4584,15 +4729,15 @@
         <v>A0104.jpg</v>
       </c>
       <c r="I108" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="109" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>17</v>
@@ -4614,15 +4759,15 @@
         <v>A0105.jpg</v>
       </c>
       <c r="I109" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="110" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>17</v>
@@ -4644,15 +4789,15 @@
         <v>A0106.jpg</v>
       </c>
       <c r="I110" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="111" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>17</v>
@@ -4674,15 +4819,15 @@
         <v>A0107.jpg</v>
       </c>
       <c r="I111" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="112" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>17</v>
@@ -4704,15 +4849,15 @@
         <v>A0108.jpg</v>
       </c>
       <c r="I112" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="113" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>17</v>
@@ -4734,15 +4879,15 @@
         <v>A0109.jpg</v>
       </c>
       <c r="I113" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="114" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>17</v>
@@ -4764,15 +4909,15 @@
         <v>A0110.jpg</v>
       </c>
       <c r="I114" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="115" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>17</v>
@@ -4794,15 +4939,15 @@
         <v>A0111.jpg</v>
       </c>
       <c r="I115" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="116" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>17</v>
@@ -4824,15 +4969,15 @@
         <v>A0112.jpg</v>
       </c>
       <c r="I116" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="117" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>17</v>
@@ -4854,15 +4999,15 @@
         <v>A0136.jpg</v>
       </c>
       <c r="I117" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="118" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>17</v>
@@ -4884,15 +5029,15 @@
         <v>A0113.jpg</v>
       </c>
       <c r="I118" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="119" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>17</v>
@@ -4914,15 +5059,15 @@
         <v>A0114.jpg</v>
       </c>
       <c r="I119" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="120" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>17</v>
@@ -4944,15 +5089,15 @@
         <v>A0115.jpg</v>
       </c>
       <c r="I120" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="121" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>17</v>
@@ -4974,15 +5119,15 @@
         <v>A0116.jpg</v>
       </c>
       <c r="I121" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="122" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A122" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>17</v>
@@ -5004,15 +5149,15 @@
         <v>A0117.jpg</v>
       </c>
       <c r="I122" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="123" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A123" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>17</v>
@@ -5034,15 +5179,15 @@
         <v>A0118.jpg</v>
       </c>
       <c r="I123" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="124" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A124" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>17</v>
@@ -5064,15 +5209,15 @@
         <v>A0119.jpg</v>
       </c>
       <c r="I124" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="125" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A125" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>17</v>
@@ -5094,15 +5239,15 @@
         <v>A0120.jpg</v>
       </c>
       <c r="I125" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="126" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A126" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>17</v>
@@ -5124,15 +5269,15 @@
         <v>A0121.jpg</v>
       </c>
       <c r="I126" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="127" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A127" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>17</v>
@@ -5154,15 +5299,15 @@
         <v>A0122.jpg</v>
       </c>
       <c r="I127" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="128" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A128" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>17</v>
@@ -5184,15 +5329,15 @@
         <v>A0123.jpg</v>
       </c>
       <c r="I128" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="129" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A129" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>17</v>
@@ -5214,15 +5359,15 @@
         <v>A0124.jpg</v>
       </c>
       <c r="I129" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="130" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A130" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>17</v>
@@ -5244,15 +5389,15 @@
         <v>A0125.jpg</v>
       </c>
       <c r="I130" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="131" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A131" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>17</v>
@@ -5274,15 +5419,15 @@
         <v>A0126.jpg</v>
       </c>
       <c r="I131" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="132" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A132" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>17</v>
@@ -5304,15 +5449,15 @@
         <v>A0127.jpg</v>
       </c>
       <c r="I132" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="133" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A133" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>17</v>
@@ -5334,15 +5479,15 @@
         <v>A0128.jpg</v>
       </c>
       <c r="I133" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="134" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A134" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>17</v>
@@ -5364,15 +5509,15 @@
         <v>A0129.jpg</v>
       </c>
       <c r="I134" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="135" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A135" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>17</v>
@@ -5394,15 +5539,15 @@
         <v>A0130.jpg</v>
       </c>
       <c r="I135" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="136" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A136" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>17</v>
@@ -5424,15 +5569,15 @@
         <v>A0131.jpg</v>
       </c>
       <c r="I136" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="137" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A137" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C137" s="1" t="s">
         <v>17</v>
@@ -5454,7 +5599,577 @@
         <v>A0132.jpg</v>
       </c>
       <c r="I137" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
+        <v>298</v>
+      </c>
+      <c r="B138" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="C138" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D138" s="14">
+        <v>560</v>
+      </c>
+      <c r="E138" s="13">
+        <v>12</v>
+      </c>
+      <c r="F138" s="13">
+        <v>12</v>
+      </c>
+      <c r="G138">
+        <v>0</v>
+      </c>
+      <c r="H138" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v>A0137.jpg</v>
+      </c>
+      <c r="I138" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
+        <v>299</v>
+      </c>
+      <c r="B139" s="10" t="s">
+        <v>305</v>
+      </c>
+      <c r="C139" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D139" s="11">
+        <v>4600</v>
+      </c>
+      <c r="E139" s="12">
+        <v>1</v>
+      </c>
+      <c r="F139" s="12">
+        <v>1</v>
+      </c>
+      <c r="G139">
+        <v>100</v>
+      </c>
+      <c r="H139" t="str">
+        <f t="shared" si="1"/>
+        <v>A0138.jpg</v>
+      </c>
+      <c r="I139" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
+        <v>300</v>
+      </c>
+      <c r="B140" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="C140" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D140" s="11">
+        <v>300</v>
+      </c>
+      <c r="E140" s="12">
+        <v>10</v>
+      </c>
+      <c r="F140" s="12">
+        <v>1</v>
+      </c>
+      <c r="G140">
+        <v>100</v>
+      </c>
+      <c r="H140" t="str">
+        <f t="shared" si="1"/>
+        <v>A0139.jpg</v>
+      </c>
+      <c r="I140" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
+        <v>301</v>
+      </c>
+      <c r="B141" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="C141" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D141" s="15">
+        <v>0</v>
+      </c>
+      <c r="E141" s="12">
+        <v>0</v>
+      </c>
+      <c r="F141" s="12">
+        <v>0</v>
+      </c>
+      <c r="G141">
+        <v>0</v>
+      </c>
+      <c r="H141" t="str">
+        <f t="shared" si="1"/>
+        <v>A0140.jpg</v>
+      </c>
+      <c r="I141" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
+        <v>302</v>
+      </c>
+      <c r="B142" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="C142" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D142">
+        <v>64</v>
+      </c>
+      <c r="E142">
+        <v>36</v>
+      </c>
+      <c r="F142">
+        <v>36</v>
+      </c>
+      <c r="G142">
+        <v>0</v>
+      </c>
+      <c r="H142" t="str">
+        <f t="shared" si="1"/>
+        <v>A0141.jpg</v>
+      </c>
+      <c r="I142" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>303</v>
+      </c>
+      <c r="B143" s="10" t="s">
+        <v>309</v>
+      </c>
+      <c r="C143" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D143">
+        <v>105</v>
+      </c>
+      <c r="E143">
+        <v>24</v>
+      </c>
+      <c r="F143">
+        <v>24</v>
+      </c>
+      <c r="G143">
+        <v>0</v>
+      </c>
+      <c r="H143" t="str">
+        <f t="shared" si="1"/>
+        <v>A0142.jpg</v>
+      </c>
+      <c r="I143" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>311</v>
+      </c>
+      <c r="B144" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="C144" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D144">
+        <v>130</v>
+      </c>
+      <c r="E144">
+        <v>25</v>
+      </c>
+      <c r="F144">
+        <v>25</v>
+      </c>
+      <c r="G144">
+        <v>100</v>
+      </c>
+      <c r="H144" t="str">
+        <f t="shared" si="1"/>
+        <v>A0143.jpg</v>
+      </c>
+      <c r="I144" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>312</v>
+      </c>
+      <c r="B145" s="10" t="s">
+        <v>319</v>
+      </c>
+      <c r="C145" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D145">
+        <v>510</v>
+      </c>
+      <c r="E145">
+        <v>10</v>
+      </c>
+      <c r="F145">
+        <v>1</v>
+      </c>
+      <c r="G145">
+        <v>100</v>
+      </c>
+      <c r="H145" t="str">
+        <f t="shared" si="1"/>
+        <v>A0144.jpg</v>
+      </c>
+      <c r="I145" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
+        <v>313</v>
+      </c>
+      <c r="B146" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="C146" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D146">
+        <v>510</v>
+      </c>
+      <c r="E146">
+        <v>10</v>
+      </c>
+      <c r="F146">
+        <v>1</v>
+      </c>
+      <c r="G146">
+        <v>100</v>
+      </c>
+      <c r="H146" t="str">
+        <f t="shared" ref="H146:H160" si="2">_xlfn.CONCAT(A146,".jpg")</f>
+        <v>A0145.jpg</v>
+      </c>
+      <c r="I146" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
+        <v>314</v>
+      </c>
+      <c r="B147" s="10" t="s">
+        <v>316</v>
+      </c>
+      <c r="C147" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D147">
+        <v>1200</v>
+      </c>
+      <c r="E147">
+        <v>5</v>
+      </c>
+      <c r="F147">
+        <v>1</v>
+      </c>
+      <c r="G147">
+        <v>100</v>
+      </c>
+      <c r="H147" t="str">
+        <f t="shared" si="2"/>
+        <v>A0146.jpg</v>
+      </c>
+      <c r="I147" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
+        <v>315</v>
+      </c>
+      <c r="B148" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="C148" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D148">
+        <v>460</v>
+      </c>
+      <c r="E148" s="15">
+        <v>0</v>
+      </c>
+      <c r="F148" s="15">
+        <v>0</v>
+      </c>
+      <c r="G148">
+        <v>0</v>
+      </c>
+      <c r="H148" t="str">
+        <f t="shared" si="2"/>
+        <v>A0147.jpg</v>
+      </c>
+      <c r="I148" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>321</v>
+      </c>
+      <c r="B149" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="C149" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D149">
+        <v>75</v>
+      </c>
+      <c r="E149">
+        <v>24</v>
+      </c>
+      <c r="F149">
+        <v>24</v>
+      </c>
+      <c r="G149">
+        <v>100</v>
+      </c>
+      <c r="H149" t="str">
+        <f t="shared" si="2"/>
+        <v>A0148.jpg</v>
+      </c>
+      <c r="I149" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>329</v>
+      </c>
+      <c r="B150" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="C150" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D150" s="15">
+        <v>0</v>
+      </c>
+      <c r="E150">
+        <v>0</v>
+      </c>
+      <c r="F150">
+        <v>0</v>
+      </c>
+      <c r="G150">
+        <v>0</v>
+      </c>
+      <c r="H150" t="str">
+        <f t="shared" si="2"/>
+        <v>A0149.jpg</v>
+      </c>
+      <c r="I150" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>330</v>
+      </c>
+      <c r="B151" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C151" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D151">
+        <v>1275</v>
+      </c>
+      <c r="E151">
+        <v>1</v>
+      </c>
+      <c r="F151">
+        <v>1</v>
+      </c>
+      <c r="G151">
+        <v>100</v>
+      </c>
+      <c r="H151" t="str">
+        <f t="shared" si="2"/>
+        <v>A0150.jpg</v>
+      </c>
+      <c r="I151" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>331</v>
+      </c>
+      <c r="B152" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="C152" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D152">
+        <v>3000</v>
+      </c>
+      <c r="E152">
+        <v>1</v>
+      </c>
+      <c r="F152">
+        <v>1</v>
+      </c>
+      <c r="G152">
+        <v>100</v>
+      </c>
+      <c r="H152" t="str">
+        <f t="shared" si="2"/>
+        <v>A0151.jpg</v>
+      </c>
+      <c r="I152" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>332</v>
+      </c>
+      <c r="B153" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="C153" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D153">
+        <v>1580</v>
+      </c>
+      <c r="E153">
+        <v>12</v>
+      </c>
+      <c r="F153">
+        <v>12</v>
+      </c>
+      <c r="G153">
+        <v>100</v>
+      </c>
+      <c r="H153" t="str">
+        <f t="shared" si="2"/>
+        <v>A0152.jpg</v>
+      </c>
+      <c r="I153" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A154" t="s">
+        <v>333</v>
+      </c>
+      <c r="B154" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="C154" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D154">
+        <v>210</v>
+      </c>
+      <c r="E154">
+        <v>10</v>
+      </c>
+      <c r="F154">
+        <v>1</v>
+      </c>
+      <c r="G154">
+        <v>100</v>
+      </c>
+      <c r="H154" t="str">
+        <f t="shared" si="2"/>
+        <v>A0153.jpg</v>
+      </c>
+      <c r="I154" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A155" t="s">
+        <v>334</v>
+      </c>
+      <c r="B155" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="C155" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D155">
+        <v>660</v>
+      </c>
+      <c r="E155">
+        <v>6</v>
+      </c>
+      <c r="F155">
+        <v>6</v>
+      </c>
+      <c r="G155">
+        <v>100</v>
+      </c>
+      <c r="H155" t="str">
+        <f t="shared" si="2"/>
+        <v>A0154.jpg</v>
+      </c>
+      <c r="I155" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>335</v>
+      </c>
+      <c r="B156" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="C156" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D156">
+        <v>1600</v>
+      </c>
+      <c r="E156">
+        <v>5</v>
+      </c>
+      <c r="F156">
+        <v>1</v>
+      </c>
+      <c r="G156">
+        <v>100</v>
+      </c>
+      <c r="H156" t="str">
+        <f t="shared" si="2"/>
+        <v>A0155.jpg</v>
+      </c>
+      <c r="I156" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Importador de Excel con normalización de categoría + fixes
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucil\Desktop\rmkits-main\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/064937db6ab52f6d/Desktop/web_carrito/rmkits/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25564EA4-A796-44CA-913D-60037C28D03E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{25564EA4-A796-44CA-913D-60037C28D03E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F878A076-516C-47E6-AAA0-D31183725283}"/>
   <bookViews>
-    <workbookView xWindow="150" yWindow="1460" windowWidth="8860" windowHeight="9820" xr2:uid="{C4B6B2E4-7AFF-45F0-BE4D-6E6AB0ED2031}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{C4B6B2E4-7AFF-45F0-BE4D-6E6AB0ED2031}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1164,7 +1164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1188,19 +1188,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1522,15 +1516,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B0D8A5A-108C-466C-953C-70B57E87E4C5}">
   <dimension ref="A1:I156"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.1796875" customWidth="1"/>
-    <col min="2" max="2" width="39.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.36328125" customWidth="1"/>
-    <col min="9" max="9" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" customWidth="1"/>
+    <col min="2" max="2" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.42578125" customWidth="1"/>
+    <col min="9" max="9" width="16.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1559,7 +1553,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1570,7 +1564,7 @@
         <v>16</v>
       </c>
       <c r="D2" s="5">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E2" s="5">
         <v>12</v>
@@ -1588,7 +1582,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1617,7 +1611,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1646,7 +1640,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1675,7 +1669,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1704,7 +1698,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1733,7 +1727,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1762,7 +1756,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1791,7 +1785,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1820,7 +1814,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>64</v>
       </c>
@@ -1849,7 +1843,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>65</v>
       </c>
@@ -1878,7 +1872,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>66</v>
       </c>
@@ -1907,7 +1901,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -1936,7 +1930,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>68</v>
       </c>
@@ -1965,7 +1959,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>69</v>
       </c>
@@ -1994,7 +1988,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>70</v>
       </c>
@@ -2024,7 +2018,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -2054,7 +2048,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>72</v>
       </c>
@@ -2084,7 +2078,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>73</v>
       </c>
@@ -2114,7 +2108,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>111</v>
       </c>
@@ -2144,7 +2138,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>74</v>
       </c>
@@ -2174,7 +2168,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>75</v>
       </c>
@@ -2204,7 +2198,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -2234,7 +2228,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>77</v>
       </c>
@@ -2264,7 +2258,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>78</v>
       </c>
@@ -2294,7 +2288,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>79</v>
       </c>
@@ -2324,7 +2318,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>80</v>
       </c>
@@ -2354,7 +2348,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>81</v>
       </c>
@@ -2384,7 +2378,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>82</v>
       </c>
@@ -2414,7 +2408,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>83</v>
       </c>
@@ -2444,7 +2438,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>84</v>
       </c>
@@ -2474,7 +2468,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>97</v>
       </c>
@@ -2504,7 +2498,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>98</v>
       </c>
@@ -2534,7 +2528,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>99</v>
       </c>
@@ -2564,7 +2558,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>100</v>
       </c>
@@ -2594,7 +2588,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>101</v>
       </c>
@@ -2624,7 +2618,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>102</v>
       </c>
@@ -2654,7 +2648,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>103</v>
       </c>
@@ -2684,7 +2678,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>104</v>
       </c>
@@ -2714,7 +2708,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>105</v>
       </c>
@@ -2744,7 +2738,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>106</v>
       </c>
@@ -2774,7 +2768,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>107</v>
       </c>
@@ -2804,7 +2798,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>108</v>
       </c>
@@ -2834,7 +2828,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>271</v>
       </c>
@@ -2862,7 +2856,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>273</v>
       </c>
@@ -2890,7 +2884,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>109</v>
       </c>
@@ -2920,7 +2914,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>110</v>
       </c>
@@ -2950,7 +2944,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>112</v>
       </c>
@@ -2978,7 +2972,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>163</v>
       </c>
@@ -3006,7 +3000,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>164</v>
       </c>
@@ -3036,7 +3030,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>165</v>
       </c>
@@ -3066,7 +3060,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>166</v>
       </c>
@@ -3096,7 +3090,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>167</v>
       </c>
@@ -3126,7 +3120,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>168</v>
       </c>
@@ -3156,7 +3150,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>169</v>
       </c>
@@ -3186,7 +3180,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>170</v>
       </c>
@@ -3216,7 +3210,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>171</v>
       </c>
@@ -3246,7 +3240,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="26" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:9" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>172</v>
       </c>
@@ -3257,7 +3251,7 @@
         <v>17</v>
       </c>
       <c r="D59" s="7">
-        <v>1700</v>
+        <v>2520</v>
       </c>
       <c r="E59" s="7">
         <v>12</v>
@@ -3276,7 +3270,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>173</v>
       </c>
@@ -3306,7 +3300,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>174</v>
       </c>
@@ -3336,7 +3330,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>175</v>
       </c>
@@ -3366,7 +3360,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>176</v>
       </c>
@@ -3396,7 +3390,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>177</v>
       </c>
@@ -3426,7 +3420,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>178</v>
       </c>
@@ -3456,7 +3450,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>179</v>
       </c>
@@ -3486,7 +3480,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:9" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>180</v>
       </c>
@@ -3516,7 +3510,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:9" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>181</v>
       </c>
@@ -3546,7 +3540,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:9" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>182</v>
       </c>
@@ -3576,7 +3570,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>183</v>
       </c>
@@ -3606,7 +3600,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>184</v>
       </c>
@@ -3636,7 +3630,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>185</v>
       </c>
@@ -3666,7 +3660,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>186</v>
       </c>
@@ -3696,7 +3690,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>187</v>
       </c>
@@ -3726,7 +3720,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>188</v>
       </c>
@@ -3756,7 +3750,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>189</v>
       </c>
@@ -3786,7 +3780,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>190</v>
       </c>
@@ -3816,7 +3810,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>191</v>
       </c>
@@ -3846,7 +3840,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>192</v>
       </c>
@@ -3876,7 +3870,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>193</v>
       </c>
@@ -3906,7 +3900,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>194</v>
       </c>
@@ -3936,7 +3930,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>281</v>
       </c>
@@ -3966,7 +3960,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>195</v>
       </c>
@@ -3996,7 +3990,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>196</v>
       </c>
@@ -4026,7 +4020,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>197</v>
       </c>
@@ -4056,7 +4050,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>198</v>
       </c>
@@ -4086,7 +4080,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>199</v>
       </c>
@@ -4116,11 +4110,11 @@
         <v>49</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>200</v>
       </c>
-      <c r="B88" s="9" t="s">
+      <c r="B88" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C88" s="1" t="s">
@@ -4146,7 +4140,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>201</v>
       </c>
@@ -4176,7 +4170,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>202</v>
       </c>
@@ -4206,7 +4200,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>203</v>
       </c>
@@ -4236,7 +4230,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>204</v>
       </c>
@@ -4266,7 +4260,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>205</v>
       </c>
@@ -4294,7 +4288,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>206</v>
       </c>
@@ -4322,7 +4316,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>207</v>
       </c>
@@ -4350,7 +4344,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>208</v>
       </c>
@@ -4378,7 +4372,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>209</v>
       </c>
@@ -4406,7 +4400,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>210</v>
       </c>
@@ -4434,7 +4428,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>211</v>
       </c>
@@ -4462,7 +4456,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>212</v>
       </c>
@@ -4492,7 +4486,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>213</v>
       </c>
@@ -4522,7 +4516,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>214</v>
       </c>
@@ -4552,7 +4546,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>215</v>
       </c>
@@ -4582,7 +4576,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>216</v>
       </c>
@@ -4612,7 +4606,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>217</v>
       </c>
@@ -4642,7 +4636,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>218</v>
       </c>
@@ -4672,7 +4666,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>219</v>
       </c>
@@ -4702,7 +4696,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>220</v>
       </c>
@@ -4732,7 +4726,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>221</v>
       </c>
@@ -4762,7 +4756,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>222</v>
       </c>
@@ -4792,7 +4786,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>223</v>
       </c>
@@ -4822,7 +4816,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>224</v>
       </c>
@@ -4852,7 +4846,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>225</v>
       </c>
@@ -4882,7 +4876,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>226</v>
       </c>
@@ -4912,7 +4906,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>227</v>
       </c>
@@ -4942,7 +4936,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>228</v>
       </c>
@@ -4972,7 +4966,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>292</v>
       </c>
@@ -5002,7 +4996,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>229</v>
       </c>
@@ -5032,7 +5026,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>230</v>
       </c>
@@ -5062,7 +5056,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>231</v>
       </c>
@@ -5092,7 +5086,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>232</v>
       </c>
@@ -5122,7 +5116,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>233</v>
       </c>
@@ -5152,7 +5146,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>234</v>
       </c>
@@ -5182,7 +5176,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="124" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>235</v>
       </c>
@@ -5212,7 +5206,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>236</v>
       </c>
@@ -5242,7 +5236,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>237</v>
       </c>
@@ -5272,7 +5266,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>238</v>
       </c>
@@ -5302,7 +5296,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="128" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>239</v>
       </c>
@@ -5332,7 +5326,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>240</v>
       </c>
@@ -5362,7 +5356,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="130" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>241</v>
       </c>
@@ -5392,7 +5386,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>242</v>
       </c>
@@ -5422,7 +5416,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>243</v>
       </c>
@@ -5452,7 +5446,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="133" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>244</v>
       </c>
@@ -5482,7 +5476,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>245</v>
       </c>
@@ -5512,7 +5506,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="135" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>246</v>
       </c>
@@ -5542,7 +5536,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="136" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>247</v>
       </c>
@@ -5572,7 +5566,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>248</v>
       </c>
@@ -5602,29 +5596,29 @@
         <v>49</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>298</v>
       </c>
-      <c r="B138" s="10" t="s">
+      <c r="B138" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="C138" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D138" s="14">
+      <c r="C138" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D138" s="12">
         <v>560</v>
       </c>
-      <c r="E138" s="13">
-        <v>12</v>
-      </c>
-      <c r="F138" s="13">
+      <c r="E138" s="8">
+        <v>12</v>
+      </c>
+      <c r="F138" s="8">
         <v>12</v>
       </c>
       <c r="G138">
         <v>0</v>
       </c>
-      <c r="H138" s="15" t="str">
+      <c r="H138" s="13" t="str">
         <f t="shared" si="1"/>
         <v>A0137.jpg</v>
       </c>
@@ -5632,23 +5626,23 @@
         <v>49</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>299</v>
       </c>
-      <c r="B139" s="10" t="s">
+      <c r="B139" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="C139" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D139" s="11">
+      <c r="C139" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D139" s="10">
         <v>4600</v>
       </c>
-      <c r="E139" s="12">
+      <c r="E139" s="11">
         <v>1</v>
       </c>
-      <c r="F139" s="12">
+      <c r="F139" s="11">
         <v>1</v>
       </c>
       <c r="G139">
@@ -5662,23 +5656,23 @@
         <v>49</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>300</v>
       </c>
-      <c r="B140" s="10" t="s">
+      <c r="B140" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="C140" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D140" s="11">
+      <c r="C140" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D140" s="10">
         <v>300</v>
       </c>
-      <c r="E140" s="12">
+      <c r="E140" s="11">
         <v>10</v>
       </c>
-      <c r="F140" s="12">
+      <c r="F140" s="11">
         <v>1</v>
       </c>
       <c r="G140">
@@ -5692,23 +5686,23 @@
         <v>49</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>301</v>
       </c>
-      <c r="B141" s="10" t="s">
+      <c r="B141" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="C141" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D141" s="15">
+      <c r="C141" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D141" s="13">
         <v>0</v>
       </c>
-      <c r="E141" s="12">
+      <c r="E141" s="11">
         <v>0</v>
       </c>
-      <c r="F141" s="12">
+      <c r="F141" s="11">
         <v>0</v>
       </c>
       <c r="G141">
@@ -5722,14 +5716,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>302</v>
       </c>
-      <c r="B142" s="10" t="s">
+      <c r="B142" s="9" t="s">
         <v>308</v>
       </c>
-      <c r="C142" s="10" t="s">
+      <c r="C142" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D142">
@@ -5752,14 +5746,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>303</v>
       </c>
-      <c r="B143" s="10" t="s">
+      <c r="B143" s="9" t="s">
         <v>309</v>
       </c>
-      <c r="C143" s="10" t="s">
+      <c r="C143" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D143">
@@ -5782,14 +5776,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>311</v>
       </c>
-      <c r="B144" s="10" t="s">
+      <c r="B144" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="C144" s="10" t="s">
+      <c r="C144" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D144">
@@ -5812,14 +5806,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>312</v>
       </c>
-      <c r="B145" s="10" t="s">
+      <c r="B145" s="9" t="s">
         <v>319</v>
       </c>
-      <c r="C145" s="10" t="s">
+      <c r="C145" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D145">
@@ -5842,14 +5836,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>313</v>
       </c>
-      <c r="B146" s="10" t="s">
+      <c r="B146" s="9" t="s">
         <v>320</v>
       </c>
-      <c r="C146" s="10" t="s">
+      <c r="C146" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D146">
@@ -5865,21 +5859,21 @@
         <v>100</v>
       </c>
       <c r="H146" t="str">
-        <f t="shared" ref="H146:H160" si="2">_xlfn.CONCAT(A146,".jpg")</f>
+        <f t="shared" ref="H146:H156" si="2">_xlfn.CONCAT(A146,".jpg")</f>
         <v>A0145.jpg</v>
       </c>
       <c r="I146" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>314</v>
       </c>
-      <c r="B147" s="10" t="s">
+      <c r="B147" s="9" t="s">
         <v>316</v>
       </c>
-      <c r="C147" s="10" t="s">
+      <c r="C147" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D147">
@@ -5902,23 +5896,23 @@
         <v>49</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>315</v>
       </c>
-      <c r="B148" s="10" t="s">
+      <c r="B148" s="9" t="s">
         <v>317</v>
       </c>
-      <c r="C148" s="10" t="s">
+      <c r="C148" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D148">
         <v>460</v>
       </c>
-      <c r="E148" s="15">
+      <c r="E148" s="13">
         <v>0</v>
       </c>
-      <c r="F148" s="15">
+      <c r="F148" s="13">
         <v>0</v>
       </c>
       <c r="G148">
@@ -5932,14 +5926,14 @@
         <v>48</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>321</v>
       </c>
-      <c r="B149" s="10" t="s">
+      <c r="B149" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="C149" s="10" t="s">
+      <c r="C149" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D149">
@@ -5962,17 +5956,17 @@
         <v>49</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>329</v>
       </c>
-      <c r="B150" s="10" t="s">
+      <c r="B150" s="9" t="s">
         <v>328</v>
       </c>
-      <c r="C150" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D150" s="15">
+      <c r="C150" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D150" s="13">
         <v>0</v>
       </c>
       <c r="E150">
@@ -5992,14 +5986,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>330</v>
       </c>
-      <c r="B151" s="10" t="s">
+      <c r="B151" s="9" t="s">
         <v>322</v>
       </c>
-      <c r="C151" s="10" t="s">
+      <c r="C151" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D151">
@@ -6022,14 +6016,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>331</v>
       </c>
-      <c r="B152" s="10" t="s">
+      <c r="B152" s="9" t="s">
         <v>323</v>
       </c>
-      <c r="C152" s="10" t="s">
+      <c r="C152" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D152">
@@ -6052,14 +6046,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>332</v>
       </c>
-      <c r="B153" s="10" t="s">
+      <c r="B153" s="9" t="s">
         <v>324</v>
       </c>
-      <c r="C153" s="10" t="s">
+      <c r="C153" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D153">
@@ -6072,7 +6066,7 @@
         <v>12</v>
       </c>
       <c r="G153">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H153" t="str">
         <f t="shared" si="2"/>
@@ -6082,14 +6076,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>333</v>
       </c>
-      <c r="B154" s="10" t="s">
+      <c r="B154" s="9" t="s">
         <v>325</v>
       </c>
-      <c r="C154" s="10" t="s">
+      <c r="C154" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D154">
@@ -6112,14 +6106,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>334</v>
       </c>
-      <c r="B155" s="10" t="s">
+      <c r="B155" s="9" t="s">
         <v>326</v>
       </c>
-      <c r="C155" s="10" t="s">
+      <c r="C155" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D155">
@@ -6142,14 +6136,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>335</v>
       </c>
-      <c r="B156" s="10" t="s">
+      <c r="B156" s="9" t="s">
         <v>327</v>
       </c>
-      <c r="C156" s="10" t="s">
+      <c r="C156" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D156">

</xml_diff>